<commit_message>
Daily slate 2026-05-23 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-22.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-22.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" t="n">
-        <v>59.5</v>
+        <v>59.8</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="5">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
         <v>12</v>
       </c>
       <c r="G6" t="n">
-        <v>50</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>60</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E8" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F8" t="n">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G8" t="n">
-        <v>29.2</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E9" t="n">
         <v>55</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G9" t="n">
-        <v>60.4</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>490</v>
+        <v>513</v>
       </c>
       <c r="E10" t="n">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="F10" t="n">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="G10" t="n">
-        <v>55.9</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="E11" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="F11" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="G11" t="n">
-        <v>60.4</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E12" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F12" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E13" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F13" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G13" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="E14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F14" t="n">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="G14" t="n">
-        <v>17.9</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,13 +848,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E15" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="G15" t="n">
         <v>20.4</v>
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G16" t="n">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2655</v>
+        <v>2790</v>
       </c>
       <c r="E17" t="n">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="F17" t="n">
-        <v>2163</v>
+        <v>2287</v>
       </c>
       <c r="G17" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1489,52 +1489,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55.9</v>
+        <v>55.2</v>
       </c>
       <c r="C7" t="n">
-        <v>490</v>
+        <v>513</v>
       </c>
       <c r="D7" t="n">
-        <v>60.4</v>
+        <v>60.1</v>
       </c>
       <c r="E7" t="n">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="F7" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="H7" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="I7" t="n">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="J7" t="n">
-        <v>17.9</v>
+        <v>17.5</v>
       </c>
       <c r="K7" t="n">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="L7" t="n">
         <v>20.4</v>
       </c>
       <c r="M7" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="N7" t="n">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="O7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P7" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="Q7" t="n">
-        <v>2655</v>
+        <v>2790</v>
       </c>
       <c r="R7" t="n">
         <v>33.3</v>
@@ -1543,28 +1543,28 @@
         <v>12</v>
       </c>
       <c r="T7" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="U7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>50</v>
+        <v>53.8</v>
       </c>
       <c r="W7" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="X7" t="n">
-        <v>29.2</v>
+        <v>29.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="Z7" t="n">
-        <v>59.5</v>
+        <v>59.8</v>
       </c>
       <c r="AA7" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="AB7" t="n">
         <v>59.3</v>
@@ -1573,16 +1573,16 @@
         <v>27</v>
       </c>
       <c r="AD7" t="n">
-        <v>60</v>
+        <v>61.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AF7" t="n">
-        <v>60.4</v>
+        <v>59.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-05-24 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-22.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-22.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G3" t="n">
-        <v>59.8</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
       </c>
       <c r="F5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>59.3</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" t="n">
         <v>12</v>
       </c>
       <c r="G6" t="n">
-        <v>53.8</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="7">
@@ -619,13 +619,13 @@
         <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>61.5</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="E8" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F8" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G8" t="n">
-        <v>29.4</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E9" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F9" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G9" t="n">
-        <v>59.1</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>513</v>
+        <v>539</v>
       </c>
       <c r="E10" t="n">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="F10" t="n">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="G10" t="n">
-        <v>55.2</v>
+        <v>54.9</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="E11" t="n">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="F11" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G11" t="n">
-        <v>60.1</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E12" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="F12" t="n">
         <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>65.09999999999999</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E13" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F13" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G13" t="n">
-        <v>52.4</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="E14" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F14" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G14" t="n">
-        <v>17.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F15" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G15" t="n">
-        <v>20.4</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>46</v>
       </c>
       <c r="G16" t="n">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2790</v>
+        <v>3006</v>
       </c>
       <c r="E17" t="n">
-        <v>503</v>
+        <v>554</v>
       </c>
       <c r="F17" t="n">
-        <v>2287</v>
+        <v>2452</v>
       </c>
       <c r="G17" t="n">
-        <v>18</v>
+        <v>18.4</v>
       </c>
     </row>
   </sheetData>
@@ -1489,52 +1489,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55.2</v>
+        <v>54.9</v>
       </c>
       <c r="C7" t="n">
-        <v>513</v>
+        <v>539</v>
       </c>
       <c r="D7" t="n">
-        <v>60.1</v>
+        <v>60.5</v>
       </c>
       <c r="E7" t="n">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="F7" t="n">
-        <v>65.09999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="G7" t="n">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H7" t="n">
-        <v>52.4</v>
+        <v>53.1</v>
       </c>
       <c r="I7" t="n">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="J7" t="n">
-        <v>17.5</v>
+        <v>20</v>
       </c>
       <c r="K7" t="n">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="L7" t="n">
-        <v>20.4</v>
+        <v>22.1</v>
       </c>
       <c r="M7" t="n">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="N7" t="n">
-        <v>8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="P7" t="n">
-        <v>18</v>
+        <v>18.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>2790</v>
+        <v>3006</v>
       </c>
       <c r="R7" t="n">
         <v>33.3</v>
@@ -1543,46 +1543,46 @@
         <v>12</v>
       </c>
       <c r="T7" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
       <c r="U7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V7" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="W7" t="n">
+        <v>27</v>
+      </c>
+      <c r="X7" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>487</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>86</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD7" t="n">
         <v>53.8</v>
-      </c>
-      <c r="W7" t="n">
-        <v>26</v>
-      </c>
-      <c r="X7" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>483</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>82</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>27</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>61.5</v>
       </c>
       <c r="AE7" t="n">
         <v>13</v>
       </c>
       <c r="AF7" t="n">
-        <v>59.1</v>
+        <v>58.8</v>
       </c>
       <c r="AG7" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>